<commit_message>
add water use efficiency per pot and figure
water_use_efficiency() divides end-point shoot dry weight (end-point sheet)
by total water added. 02_join_metadata.R adds it to water_added_per_pot.xlsx
and plots it by treatment. endpoint_sheet is now a required config entry.
</commit_message>
<xml_diff>
--- a/output/tables/water_added_per_pot.xlsx
+++ b/output/tables/water_added_per_pot.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
@@ -408,6 +408,16 @@
           <t>Water_Total_g</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Shoot_Dry_Weight_mg</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>WUE_mg_per_g</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -445,6 +455,12 @@
       <c r="I2">
         <v>2616</v>
       </c>
+      <c r="J2">
+        <v>2596.6</v>
+      </c>
+      <c r="K2">
+        <v>0.9925840978593272</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -482,6 +498,12 @@
       <c r="I3">
         <v>2441</v>
       </c>
+      <c r="J3">
+        <v>2177.3</v>
+      </c>
+      <c r="K3">
+        <v>0.8919705038918477</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -519,6 +541,12 @@
       <c r="I4">
         <v>2562</v>
       </c>
+      <c r="J4">
+        <v>2256</v>
+      </c>
+      <c r="K4">
+        <v>0.8805620608899297</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -556,6 +584,12 @@
       <c r="I5">
         <v>2406</v>
       </c>
+      <c r="J5">
+        <v>2001.2</v>
+      </c>
+      <c r="K5">
+        <v>0.8317539484621779</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -593,6 +627,12 @@
       <c r="I6">
         <v>2087</v>
       </c>
+      <c r="J6">
+        <v>611</v>
+      </c>
+      <c r="K6">
+        <v>0.2927647340680403</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -630,6 +670,12 @@
       <c r="I7">
         <v>2101</v>
       </c>
+      <c r="J7">
+        <v>756</v>
+      </c>
+      <c r="K7">
+        <v>0.3598286530223703</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -667,6 +713,12 @@
       <c r="I8">
         <v>2752</v>
       </c>
+      <c r="J8">
+        <v>2639.1</v>
+      </c>
+      <c r="K8">
+        <v>0.9589752906976744</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -704,6 +756,12 @@
       <c r="I9">
         <v>2621</v>
       </c>
+      <c r="J9">
+        <v>2133.3</v>
+      </c>
+      <c r="K9">
+        <v>0.8139259824494468</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -741,6 +799,12 @@
       <c r="I10">
         <v>2721</v>
       </c>
+      <c r="J10">
+        <v>2354.5</v>
+      </c>
+      <c r="K10">
+        <v>0.8653068724733554</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -778,6 +842,12 @@
       <c r="I11">
         <v>2525</v>
       </c>
+      <c r="J11">
+        <v>2202.4</v>
+      </c>
+      <c r="K11">
+        <v>0.8722376237623762</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -815,6 +885,12 @@
       <c r="I12">
         <v>2161</v>
       </c>
+      <c r="J12">
+        <v>742.6</v>
+      </c>
+      <c r="K12">
+        <v>0.3436372049976862</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -852,6 +928,12 @@
       <c r="I13">
         <v>2184</v>
       </c>
+      <c r="J13">
+        <v>695.1</v>
+      </c>
+      <c r="K13">
+        <v>0.3182692307692308</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -889,6 +971,12 @@
       <c r="I14">
         <v>2283</v>
       </c>
+      <c r="J14">
+        <v>1953.6</v>
+      </c>
+      <c r="K14">
+        <v>0.8557161629434954</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -926,6 +1014,12 @@
       <c r="I15">
         <v>2299</v>
       </c>
+      <c r="J15">
+        <v>1882.6</v>
+      </c>
+      <c r="K15">
+        <v>0.8188777729447585</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -963,6 +1057,12 @@
       <c r="I16">
         <v>2323</v>
       </c>
+      <c r="J16">
+        <v>1858.6</v>
+      </c>
+      <c r="K16">
+        <v>0.8000860955660783</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1000,6 +1100,12 @@
       <c r="I17">
         <v>2213</v>
       </c>
+      <c r="J17">
+        <v>1564.7</v>
+      </c>
+      <c r="K17">
+        <v>0.707049254405784</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1037,6 +1143,12 @@
       <c r="I18">
         <v>2165</v>
       </c>
+      <c r="J18">
+        <v>690.6</v>
+      </c>
+      <c r="K18">
+        <v>0.3189838337182448</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1074,6 +1186,12 @@
       <c r="I19">
         <v>2159</v>
       </c>
+      <c r="J19">
+        <v>315.1</v>
+      </c>
+      <c r="K19">
+        <v>0.1459471977767485</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1111,6 +1229,12 @@
       <c r="I20">
         <v>2328</v>
       </c>
+      <c r="J20">
+        <v>2054.4</v>
+      </c>
+      <c r="K20">
+        <v>0.8824742268041238</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1148,6 +1272,12 @@
       <c r="I21">
         <v>2264</v>
       </c>
+      <c r="J21">
+        <v>1531</v>
+      </c>
+      <c r="K21">
+        <v>0.6762367491166078</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1185,6 +1315,12 @@
       <c r="I22">
         <v>2353</v>
       </c>
+      <c r="J22">
+        <v>1696.7</v>
+      </c>
+      <c r="K22">
+        <v>0.7210794730131747</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1222,6 +1358,12 @@
       <c r="I23">
         <v>2307</v>
       </c>
+      <c r="J23">
+        <v>1567.2</v>
+      </c>
+      <c r="K23">
+        <v>0.6793237971391418</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1259,6 +1401,12 @@
       <c r="I24">
         <v>2125</v>
       </c>
+      <c r="J24">
+        <v>511.8</v>
+      </c>
+      <c r="K24">
+        <v>0.2408470588235294</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1295,6 +1443,12 @@
       </c>
       <c r="I25">
         <v>2131</v>
+      </c>
+      <c r="J25">
+        <v>484.4</v>
+      </c>
+      <c r="K25">
+        <v>0.2273111215391835</v>
       </c>
     </row>
   </sheetData>

</xml_diff>